<commit_message>
Update GTENG-15832 traceability evidence package
</commit_message>
<xml_diff>
--- a/tables/Article 127 tables.xlsx
+++ b/tables/Article 127 tables.xlsx
@@ -15,6 +15,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External trend validation" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limiting cases" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Table 4 Demand Cases" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Table 5 Validation" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Table 6 AE Evidence" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Table 7 Decisions" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Addition" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,15 +41,20 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -58,14 +68,34 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -710,6 +740,436 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Evidence stream</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>What it checks</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Main implication</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Published footing/load-settlement response</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>MICP can improve stiffness and bearing response at footing scale.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Initial improvement is physically plausible but must be linked to durability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Durability-retention evidence</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Cementation benefit can decay under exposure and ageing.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Permanent credit is not defensible without retention evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Limit-analysis and FEM checks</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Treatment-depth benefit is monotonic but bounded.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Depth credit should saturate and should not replace site-specific analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Reproducible benchmark scripts</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Capacity, beta, serviceability, and redesign outputs can be regenerated.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>The workflow is auditable rather than a single opaque example.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>AE concern</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Evidence basis</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Use in model</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Claim boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Cohesion and friction degradation</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Kulkarni et al. 2021 PLT/UCS ranges; de Rezende et al. 2022 and Gao et al. 2019 triaxial component behavior; local anti-double-counting audit.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Bounds cb0_prime, Delta tan phi, and eta(t) as component-constrained inputs.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Not a universal footing-scale cohesion/friction degradation law.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Residual cementation and degradation clock</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Ahenkorah et al. 2023 durability tests and Sharma et al. 2021 retention data in the supplemental calibration files.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Provides exposure-clock priors for eta_r and lambda_E.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Calendar-year lambda_e requires environmental-history updating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Treated-zone contribution</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>PLT response, open-source limit analysis, OpenSeesPy, and CalculiX virtual footing audits.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Supports a capped H/B screening function and treated-depth sensitivity.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Not an experimentally calibrated physical H/B law for MICP footing layers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Localization fragility</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>No direct post-peak localization data are available in the present evidence package.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>chi_s is retained only as a sensitivity and falsification factor.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>chi_s is not identified experimentally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Time-dependent capacity outcomes</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Component-calibrated parameters, model hierarchy ablation, and V0-V4 validation scale.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Supports scenario predictions and design updating.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>No direct degraded-footing V5 validation is claimed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Use in design</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Action if unfavorable</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>beta(t), pf(t)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Checks time-dependent ultimate reliability.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Reduce demand, improve treatment, or require more verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>qservice,max</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Converts reliability target into allowable service pressure.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Resize foundation or lower service load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Serviceability index</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Flags stiffness-loss and settlement-risk screening.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Use load-settlement testing or serviceability FEM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Capping / H/B status</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Prevents unrealistic credit for thin or saturated depth effects.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Use layered limit analysis or site-specific FEM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Monitoring/update flag</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Identifies when new data should update lambda or eta_r.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Retest, monitor, or recalibrate before final design.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Citation key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Full reference</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Reason for addition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>de Rezende et al. 2022</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>de Rezende, I. M., Prietto, P. D. M., Thomé, A., and Dalla Rosa, F. (2022). Mechanical behavior of microbially induced calcite precipitation cemented sand. Geotechnical and Geological Engineering, 40(4), 1997-2008. https://doi.org/10.1007/s10706-021-02006-4</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Cited in Main Table 6 evidence-to-parameter map.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2069,4 +2529,134 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Lower-demand case</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>High-demand stress test</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Design interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>qservice</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>500 kPa</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>900-950 kPa</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Demand level controls whether degraded MICP credit remains usable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>50-year FS</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>1.39</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>The high-demand case fails the usual deterministic margin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>50-year beta</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>3.96</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Reliability separates acceptable screening use from unsupported permanent credit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Serviceability index at 50 yr</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>0.0319</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0.0574</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Serviceability can become controlling before ultimate resistance is exhausted.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>